<commit_message>
redacció models + clus
</commit_message>
<xml_diff>
--- a/control_TFG.xlsx
+++ b/control_TFG.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edurne\Downloads\TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743745AD-D301-4435-9BFC-888DE666763C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2CC421-697B-402C-B6F2-35C8BAD2090A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="4440" windowWidth="20730" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -611,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -647,6 +647,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="16" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1729,15 +1732,25 @@
       <c r="C31" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="7"/>
+      <c r="D31" s="11">
+        <v>46194</v>
+      </c>
+      <c r="E31" s="11">
+        <v>46194</v>
+      </c>
+      <c r="F31" s="11">
+        <v>46194</v>
+      </c>
+      <c r="G31" s="13">
+        <v>46194</v>
+      </c>
       <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
+      <c r="I31" s="11">
+        <v>46194</v>
+      </c>
       <c r="J31" s="8"/>
       <c r="K31" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>